<commit_message>
Carrusel de fotos en las fichas del catálogo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/catalogo-mera-cake.xlsx
+++ b/plantillas/catalogo-mera-cake.xlsx
@@ -78,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -87,6 +87,7 @@
     <xf numFmtId="49" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -699,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -776,7 +777,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Foto (enlace Drive): el enlace de compartir de una foto en Google Drive.</t>
+          <t>Foto (enlace Drive): el enlace de compartir de una o varias fotos en Google Drive. Varias fotos forman un carrusel.</t>
         </is>
       </c>
     </row>
@@ -797,32 +798,39 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   · Vacío: se mantiene la foto que ya tiene la página (o el hueco, si no tiene).</t>
+          <t xml:space="preserve">   · Varias fotos: pega los enlaces en la misma celda separados por un espacio o una coma.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr"/>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   · Las fotos de la hoja se añaden después de las que ya tiene la página. Vacío: quedan solo las de la página (o el hueco).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Borrar una fila de un producto nuevo lo quita de la página. Los 4 productos fijos siguen en la página aunque</t>
-        </is>
-      </c>
+      <c r="A18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>Borrar una fila de un producto nuevo lo quita de la página. Los 4 productos fijos siguen en la página aunque</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>borres su fila (están escritos en ella para Google); para quitarlos, pídelo.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Los cambios se ven en la página al recargarla, en uno o dos minutos.</t>
         </is>

</xml_diff>